<commit_message>
minor bug fix in export/import_watchlist_from_excel
</commit_message>
<xml_diff>
--- a/watchlist.xlsx
+++ b/watchlist.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="watchlist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="watchlist" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,21 +471,29 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tim Tam</t>
+          <t>Glow Lab</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>tim tam</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Original,Deluxe</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+          <t>glow lab</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>800-1000</t>
+        </is>
+      </c>
       <c r="I2" t="b">
         <v>1</v>
       </c>
@@ -496,19 +504,32 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Kettle</t>
+          <t>old gold</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Kettle Chips</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>140-800</t>
+          <t>old gold cadbury</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>block</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
       <c r="I3" t="b">
@@ -521,19 +542,32 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Glow Lab</t>
+          <t>My Dog</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>glow lab</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+          <t>my dog</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>800-1000</t>
+          <t>350-450</t>
         </is>
       </c>
       <c r="I4" t="b">
@@ -546,25 +580,29 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>red rock</t>
+          <t>Pedigree</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>red rock</t>
+          <t>pedigree</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>chips</t>
+          <t>wet</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>lunchbox,cracker</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="I5" t="b">
         <v>1</v>
       </c>
@@ -575,21 +613,29 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>old gold</t>
+          <t>natures gift</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>old gold cadbury</t>
+          <t>natures gift</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>block</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+          <t>wet</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="I6" t="b">
         <v>1</v>
       </c>
@@ -600,24 +646,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>My Dog</t>
+          <t>bickfords</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>my dog</t>
+          <t>bickfords cordial</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>adult</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>350-450</t>
+          <t>Lemon,Ginger,Blackcurrrant</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>[]</t>
         </is>
       </c>
       <c r="I7" t="b">
@@ -630,21 +679,29 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Pedigree</t>
+          <t>Pics</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>pedigree</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>wet</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
+          <t>Pics peanut</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>350-1200</t>
+        </is>
+      </c>
       <c r="I8" t="b">
         <v>1</v>
       </c>
@@ -655,21 +712,29 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>natures gift</t>
+          <t>Mayvers</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>natures gift</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>wet</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
+          <t>Mayvers peanut</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>300-1200</t>
+        </is>
+      </c>
       <c r="I9" t="b">
         <v>1</v>
       </c>
@@ -680,21 +745,34 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>bickfords</t>
+          <t>Tim Tam</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>bickfords cordial</t>
+          <t>tim tam</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Lemon,Ginger,Blackcurrrant</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
+          <t>Original,Deluxe</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="I10" t="b">
         <v>1</v>
       </c>
@@ -705,19 +783,27 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Pics</t>
+          <t>Kettle</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Pics peanut</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+          <t>Kettle Chips</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>350-1200</t>
+          <t>140-800</t>
         </is>
       </c>
       <c r="I11" t="b">
@@ -730,25 +816,66 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mayvers</t>
+          <t>red rock</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Mayvers peanut</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>300-1200</t>
+          <t>red rock</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>chips</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>lunchbox,cracker</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>[]</t>
         </is>
       </c>
       <c r="I12" t="b">
         <v>1</v>
       </c>
       <c r="J12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Uncle Tobys</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>uncle tobys</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>iron</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="I13" t="b">
+        <v>1</v>
+      </c>
+      <c r="J13" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>